<commit_message>
research: apply course element review feedback and distinguish technical behavior interfaces
</commit_message>
<xml_diff>
--- a/stage4_course_extraction/output/03_课程知识技能点规范化表.xlsx
+++ b/stage4_course_extraction/output/03_课程知识技能点规范化表.xlsx
@@ -10,11 +10,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="规范化知识技能点" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目出现记录" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="目标及思政单列提及" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="技术行为接口" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'规范化知识技能点'!$A$1:$N$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'项目出现记录'!$A$1:$L$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'规范化知识技能点'!$A$1:$N$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'项目出现记录'!$A$1:$M$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'目标及思政单列提及'!$A$1:$K$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'技术行为接口'!$A$1:$Q$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N60"/>
+  <dimension ref="A1:N61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1573,7 +1575,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>P03;P07</t>
+          <t>P03</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1583,7 +1585,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>CE05-d0544abce4;CE11-dcbb4b95a2</t>
+          <t>CE05-d0544abce4</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1593,14 +1595,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>5;11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>CREATE TABLE
-——
-在 CREATE TABLE 时通过约束或指定索引方式创建索引。</t>
+          <t>CREATE TABLE</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -4456,286 +4456,286 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>CK060</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>建表时定义索引</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>在 CREATE TABLE 时通过约束或指定索引方式创建索引。</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>数据库管理与安全</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>按技术对象组织，非岗位证据等级或重要性排序</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>单一主要技术功能</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>P07</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>原文明示内容；名称及功能标签为研究规范化</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>CE11-dcbb4b95a2</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>在 CREATE TABLE 时通过约束或指定索引方式创建索引。</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>待审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
           <t>CK055</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B57" t="inlineStr">
         <is>
           <t>索引删除与维护</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>索引删
 除及维护</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>数据库管理与安全</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>按技术对象组织，非岗位证据等级或重要性排序</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>单一主要技术功能</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>P07</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>原文明示内容；名称及功能标签为研究规范化</t>
         </is>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I57" t="inlineStr">
         <is>
           <t>CE11-c0aa5639a8</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
-      <c r="K56" t="inlineStr">
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="L56" t="inlineStr">
+      <c r="L57" t="inlineStr">
         <is>
           <t>索引删
 除及维护</t>
         </is>
       </c>
-      <c r="M56" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
-      <c r="N56" t="inlineStr">
-        <is>
-          <t>待审查</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>待审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>CK056</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>索引查询效果对比</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>引导
 学生对比有无索引的查询效果</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>数据库管理与安全;SQL查询与数据应用</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>按技术对象组织，非岗位证据等级或重要性排序</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>同一技术作用于定义/操作与查询，或兼有概念/管理功能</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>P07</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>原文明示内容；名称及功能标签为研究规范化</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I58" t="inlineStr">
         <is>
           <t>CE11-eeed49a9bf</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
-      <c r="K57" t="inlineStr">
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="L57" t="inlineStr">
+      <c r="L58" t="inlineStr">
         <is>
           <t>引导
 学生对比有无索引的查询效果</t>
         </is>
       </c>
-      <c r="M57" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
-      <c r="N57" t="inlineStr">
-        <is>
-          <t>待审查</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>待审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
         <is>
           <t>CK057</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>数据库备份与恢复</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>数据备份与恢复的必要性。使用数据库工具或命令进行备份与恢复的基本操
 作流程。</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>数据库管理与安全</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>按技术对象组织，非岗位证据等级或重要性排序</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>单一主要技术功能</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>P08</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t>原文明示内容；名称及功能标签为研究规范化</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I59" t="inlineStr">
         <is>
           <t>CE12-f64363af28</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
-      <c r="K58" t="inlineStr">
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="L58" t="inlineStr">
+      <c r="L59" t="inlineStr">
         <is>
           <t>数据备份与恢复的必要性。使用数据库工具或命令进行备份与恢复的基本操
 作流程。</t>
         </is>
       </c>
-      <c r="M58" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
-      <c r="N58" t="inlineStr">
-        <is>
-          <t>待审查</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>CK058</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>事务概念与ACID</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>事务的概念、ACID 特性（原子性、一致性、隔离性、持久性）</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>数据库管理与安全</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>按技术对象组织，非岗位证据等级或重要性排序</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>单一主要技术功能</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>P08</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>原文明示内容；名称及功能标签为研究规范化</t>
-        </is>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>CE12-1c61fa29af</t>
-        </is>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>事务的概念、ACID 特性（原子性、一致性、隔离性、持久性）</t>
-        </is>
-      </c>
       <c r="M59" t="inlineStr">
         <is>
           <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
@@ -4750,79 +4750,151 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>CK058</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>事务概念与ACID</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>事务的概念、ACID 特性（原子性、一致性、隔离性、持久性）</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>数据库管理与安全</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>按技术对象组织，非岗位证据等级或重要性排序</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>单一主要技术功能</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>原文明示内容；名称及功能标签为研究规范化</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>CE12-1c61fa29af</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>事务的概念、ACID 特性（原子性、一致性、隔离性、持久性）</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>待审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>CK059</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>事务控制语句</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>事务
 控制语句（BEGIN, COMMIT, ROLLBACK）的使用。</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>SQL数据定义与操作;数据库管理与安全</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>按技术对象组织，非岗位证据等级或重要性排序</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>同一技术作用于定义/操作与查询，或兼有概念/管理功能</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>P08</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
+      <c r="H61" t="inlineStr">
         <is>
           <t>原文明示内容；名称及功能标签为研究规范化</t>
         </is>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="I61" t="inlineStr">
         <is>
           <t>CE12-5215a91fe3</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
-      <c r="K60" t="inlineStr">
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="L60" t="inlineStr">
+      <c r="L61" t="inlineStr">
         <is>
           <t>事务
 控制语句（BEGIN, COMMIT, ROLLBACK）的使用。</t>
         </is>
       </c>
-      <c r="M60" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
-      <c r="N60" t="inlineStr">
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N60"/>
+  <autoFilter ref="A1:N61"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4833,7 +4905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L62"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4848,6 +4920,7 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4873,40 +4946,45 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>应用语境标签</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>项目语境原文</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>知识点去重说明</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>证据ID</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>来源文件名</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>PDF实际页码</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>原文摘录</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>来源状态</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>研究者审查状态</t>
         </is>
@@ -4935,40 +5013,45 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>理解数据、数据库、数据库管理系统（DBMS）、数据库系统的概念。</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>CE03-3abb37b0df</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>理解数据、数据库、数据库管理系统（DBMS）、数据库系统的概念。</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -4997,42 +5080,47 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>了解
 数据库技术的发展及SQL 语言的基本作用。</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>CE03-832a5cc68c</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>了解
 数据库技术的发展及SQL 语言的基本作用。</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5061,40 +5149,45 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>SQL 语言的基本作用</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>CE03-5fec97ed60</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>SQL 语言的基本作用</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5123,42 +5216,47 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>掌握MySQL 安装、配置及基本连
 接方法。</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>CE03-7779270b55</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>掌握MySQL 安装、配置及基本连
 接方法。</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5187,40 +5285,45 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>数据库系统结构的理解</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>CE04-499220bd1e</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>数据库系统结构的理解</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5249,40 +5352,45 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>安装过程中错误排查与环境变量配置</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>CE04-822ed1d2cb</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>安装过程中错误排查与环境变量配置</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5311,42 +5419,47 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>树立规范操作与数据安
 全意识</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>CE04-e74f9c469f</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>树立规范操作与数据安
 全意识</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L8" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5375,40 +5488,45 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>概念模型、E-R 图、掌握概念模型、E-R 图设计及关系模式转换方法。</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>CE04-83817df1a5</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>概念模型、E-R 图、掌握概念模型、E-R 图设计及关系模式转换方法。</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5437,40 +5555,45 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>关系模式转换方法</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>CE04-f08e3fa076</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>关系模式转换方法</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5499,42 +5622,47 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>数据
 库设计规范化理论(1NF、2NF、3NF)。</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>CE04-faa84c842b</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>数据
 库设计规范化理论(1NF、2NF、3NF)。</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5563,42 +5691,47 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>数据加工、数据模型、概念模型和关系模型
 的理论</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>CE04-36d75f1fa3</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>数据加工、数据模型、概念模型和关系模型
 的理论</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5627,40 +5760,45 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>实体、属性、联系的识别与设计方法</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>CE05-ac9a866646</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>实体、属性、联系的识别与设计方法</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5689,42 +5827,47 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>在实际设计中如何平衡规范化
 与性能</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>CE05-4480d78410</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>在实际设计中如何平衡规范化
 与性能</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L14" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5753,40 +5896,45 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>CREATE DATABASE</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>CE05-ff9baef7ea</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="K15" t="inlineStr">
         <is>
           <t>CREATE DATABASE</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L15" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5815,40 +5963,45 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>数据表创建：技术对象为表结构</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>CREATE TABLE</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="G16" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
+      <c r="H16" t="inlineStr">
         <is>
           <t>CE05-d0544abce4</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="K16" t="inlineStr">
         <is>
           <t>CREATE TABLE</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5877,40 +6030,45 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>ALTER TABLE</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="G17" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>CE05-79d53429a9</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="K17" t="inlineStr">
         <is>
           <t>ALTER TABLE</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -5939,42 +6097,47 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>DROP 
 TABLE</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="G18" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="H18" t="inlineStr">
         <is>
           <t>CE05-f09aa1151b</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="K18" t="inlineStr">
         <is>
           <t>DROP 
 TABLE</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6003,40 +6166,45 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>数据完整性概念及分类（实体完整性、参照完整性、用户自定义完整性）</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="G19" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="H19" t="inlineStr">
         <is>
           <t>CE05-84b410bc0b</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="K19" t="inlineStr">
         <is>
           <t>数据完整性概念及分类（实体完整性、参照完整性、用户自定义完整性）</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L19" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6065,40 +6233,45 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>主键（PRIMARY KEY）</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="H20" t="inlineStr">
         <is>
           <t>CE05-063631ec59</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="K20" t="inlineStr">
         <is>
           <t>主键（PRIMARY KEY）</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L20" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6127,40 +6300,45 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>唯一键（UNIQUE）</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>CE05-1f52f92edd</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>唯一键（UNIQUE）</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6189,40 +6367,45 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>外键（FOREIGN KEY）</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="G22" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>CE05-be29f7a0e3</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr">
+      <c r="K22" t="inlineStr">
         <is>
           <t>外键（FOREIGN KEY）</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L22" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6251,42 +6434,47 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>检查
 约束（CHECK）</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="H23" t="inlineStr">
         <is>
           <t>CE05-8ef4ec36c4</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr">
+      <c r="K23" t="inlineStr">
         <is>
           <t>检查
 约束（CHECK）</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L23" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6315,40 +6503,45 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>数据库管理基本原则：包括命名规范、结构设计与数据安全。</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="G24" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="H24" t="inlineStr">
         <is>
           <t>CE06-66db77bb94</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="K24" t="inlineStr">
         <is>
           <t>数据库管理基本原则：包括命名规范、结构设计与数据安全。</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L24" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6377,40 +6570,45 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>命令行与图形化操作的对应关系</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="H25" t="inlineStr">
         <is>
           <t>CE06-9846220180</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I25" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
           <t>6</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>命令行与图形化操作的对应关系</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L25" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6439,42 +6637,47 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>INSERT INTO 语句的基本语法与变体（插入完整行、指定列插入、批量插
 入）</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="G26" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
+      <c r="H26" t="inlineStr">
         <is>
           <t>CE07-9ec8bc4a81</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I26" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr">
+      <c r="K26" t="inlineStr">
         <is>
           <t>INSERT INTO 语句的基本语法与变体（插入完整行、指定列插入、批量插
 入）</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6503,40 +6706,45 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>UPDATE 语句的语法结构与执行逻辑</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>CE07-aeb6f162cd</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I27" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr">
+      <c r="K27" t="inlineStr">
         <is>
           <t>UPDATE 语句的语法结构与执行逻辑</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6565,42 +6773,47 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>数据操作条件范围控制；原文明确UPDATE，删除为条件删除任务语境，不能冒称该句明示DELETE WHERE</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>WHERE 子句在精确控制更新范围
 中的关键作用</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>CE07-e21cab2f64</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I28" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr">
+      <c r="K28" t="inlineStr">
         <is>
           <t>WHERE 子句在精确控制更新范围
 中的关键作用</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6629,40 +6842,45 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>CE07-65daeb378b</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I29" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>DELETE</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L29" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6691,40 +6909,45 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>TRUNCATE TABLE</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="G30" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="H30" t="inlineStr">
         <is>
           <t>CE07-45a617ba65</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I30" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="K30" t="inlineStr">
         <is>
           <t>TRUNCATE TABLE</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L30" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6753,40 +6976,45 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>对比DELETE 与TRUNCATE 核心区别</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="G31" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr">
+      <c r="H31" t="inlineStr">
         <is>
           <t>CE07-8dd78d81d2</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I31" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr">
+      <c r="K31" t="inlineStr">
         <is>
           <t>对比DELETE 与TRUNCATE 核心区别</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L31" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6815,40 +7043,45 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>强调数据操作顺序、事务逻辑及操作安全性。</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="H32" t="inlineStr">
         <is>
           <t>CE07-e989cb5e4d</t>
         </is>
       </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I32" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr">
+      <c r="K32" t="inlineStr">
         <is>
           <t>强调数据操作顺序、事务逻辑及操作安全性。</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6877,40 +7110,45 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
           <t>SELECT 语句的基本结构</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr">
+      <c r="H33" t="inlineStr">
         <is>
           <t>CE08-37406530f3</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I33" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr">
+      <c r="K33" t="inlineStr">
         <is>
           <t>SELECT 语句的基本结构</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L33" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -6939,40 +7177,45 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>列选择（包括使用别名、表达式）</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>CE08-af736986c8</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I34" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr">
+      <c r="K34" t="inlineStr">
         <is>
           <t>列选择（包括使用别名、表达式）</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7001,42 +7244,47 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t>SELECT条件过滤：比较、逻辑与LIKE条件表达</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>WHERE 子
 句中使用比较运算符、逻辑运算符及模糊匹配（LIKE）进行条件过滤。</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="G35" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr">
+      <c r="H35" t="inlineStr">
         <is>
           <t>CE08-1b199ad8c1</t>
         </is>
       </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I35" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr">
+      <c r="K35" t="inlineStr">
         <is>
           <t>WHERE 子
 句中使用比较运算符、逻辑运算符及模糊匹配（LIKE）进行条件过滤。</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L35" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7065,40 +7313,45 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>模糊匹配（LIKE）</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="G36" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr">
+      <c r="H36" t="inlineStr">
         <is>
           <t>CE08-d1619a30d6</t>
         </is>
       </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I36" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr">
+      <c r="K36" t="inlineStr">
         <is>
           <t>模糊匹配（LIKE）</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7127,42 +7380,47 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t>连接查询
 （内连接、外连接）的原理与语法</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>CE08-149f219bac</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I37" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>连接查询
 （内连接、外连接）的原理与语法</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L37" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7191,40 +7449,45 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
           <t>子查询的概念与应用场景</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="H38" t="inlineStr">
         <is>
           <t>CE08-3d7151d36c</t>
         </is>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I38" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr">
+      <c r="K38" t="inlineStr">
         <is>
           <t>子查询的概念与应用场景</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L38" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7253,42 +7516,47 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
           <t>常用聚合函数
 （COUNT, SUM, AVG, MAX, MIN）的作用</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>CE08-ddbe4ad352</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I39" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>常用聚合函数
 （COUNT, SUM, AVG, MAX, MIN）的作用</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L39" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7317,42 +7585,47 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>GROUP BY 子句与HAVING 子句
 的配合使用</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="G40" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>CE08-7d052764f2</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I40" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="K40" t="inlineStr">
         <is>
           <t>GROUP BY 子句与HAVING 子句
 的配合使用</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7381,42 +7654,47 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>HAVING 子句
 的配合使用</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="G41" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>CE08-a7b30868fd</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I41" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="K41" t="inlineStr">
         <is>
           <t>HAVING 子句
 的配合使用</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L41" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7445,40 +7723,45 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>ORDER BY 子句排序规则</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="G42" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="H42" t="inlineStr">
         <is>
           <t>CE08-ff08dbda04</t>
         </is>
       </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I42" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="K42" t="inlineStr">
         <is>
           <t>ORDER BY 子句排序规则</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L42" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7507,42 +7790,47 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
           <t>LIMIT 子句对结果集进行分页或限定
 行数</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="G43" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>CE08-b87325ccfa</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I43" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="K43" t="inlineStr">
         <is>
           <t>LIMIT 子句对结果集进行分页或限定
 行数</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L43" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7571,40 +7859,45 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
           <t>讲解多表查询方法：JOIN、子查询、联合查询。</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="G44" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="H44" t="inlineStr">
         <is>
           <t>CE08-7f2f04d349</t>
         </is>
       </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I44" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="K44" t="inlineStr">
         <is>
           <t>讲解多表查询方法：JOIN、子查询、联合查询。</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L44" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7633,40 +7926,45 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
           <t>WHERE vs HAVING 的区别与选用</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="H45" t="inlineStr">
         <is>
           <t>CE09-ce9c0a842e</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I45" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="K45" t="inlineStr">
         <is>
           <t>WHERE vs HAVING 的区别与选用</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L45" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7695,40 +7993,45 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>分析语句执行顺序</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>CE09-a437cb96db</t>
         </is>
       </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I46" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="K46" t="inlineStr">
         <is>
           <t>分析语句执行顺序</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L46" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7757,40 +8060,45 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
           <t>强调数据隐私保护意识</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="G47" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="H47" t="inlineStr">
         <is>
           <t>CE09-a4b307e3fb</t>
         </is>
       </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I47" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="K47" t="inlineStr">
         <is>
           <t>强调数据隐私保护意识</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L47" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7819,40 +8127,45 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>视图的概念、作用与虚拟表的本质</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="G48" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="H48" t="inlineStr">
         <is>
           <t>CE09-fc942d7775</t>
         </is>
       </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I48" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr">
+      <c r="K48" t="inlineStr">
         <is>
           <t>视图的概念、作用与虚拟表的本质</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7881,42 +8194,47 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
           <t>创建视图（CREATE VIEW）的语法与
 选项</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="H49" t="inlineStr">
         <is>
           <t>CE09-3ca366e6c5</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I49" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr">
+      <c r="K49" t="inlineStr">
         <is>
           <t>创建视图（CREATE VIEW）的语法与
 选项</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L49" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -7945,40 +8263,45 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>查询视图与查询基表的异同</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>CE09-33f1ee4875</t>
         </is>
       </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I50" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>查询视图与查询基表的异同</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L50" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8007,42 +8330,47 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
           <t>通过视图进行数据插入、更新与删除的条件
 与限制</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="H51" t="inlineStr">
         <is>
           <t>CE09-0652636103</t>
         </is>
       </c>
-      <c r="H51" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I51" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr">
+      <c r="K51" t="inlineStr">
         <is>
           <t>通过视图进行数据插入、更新与删除的条件
 与限制</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L51" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8071,40 +8399,45 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
           <t>修改（ALTER VIEW）</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="G52" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>CE09-3caa03859a</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I52" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr">
+      <c r="K52" t="inlineStr">
         <is>
           <t>修改（ALTER VIEW）</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L52" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8133,42 +8466,47 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
           <t>删除（DROP VIEW）视图定义的语法及其对
 数据的影响</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="H53" t="inlineStr">
         <is>
           <t>CE09-96f297c62c</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I53" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
           <t>9</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr">
+      <c r="K53" t="inlineStr">
         <is>
           <t>删除（DROP VIEW）视图定义的语法及其对
 数据的影响</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L53" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8197,42 +8535,47 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
           <t>索引的概念、作用。常见索引类型（如普通索引、唯一索引、主键索引等）
 及其适用场景。</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="H54" t="inlineStr">
         <is>
           <t>CE11-e133c6fc3e</t>
         </is>
       </c>
-      <c r="H54" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I54" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
           <t>11</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr">
+      <c r="K54" t="inlineStr">
         <is>
           <t>索引的概念、作用。常见索引类型（如普通索引、唯一索引、主键索引等）
 及其适用场景。</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L54" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8261,40 +8604,45 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
           <t>使用 CREATE INDEX 语句创建索引</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="G55" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr">
+      <c r="H55" t="inlineStr">
         <is>
           <t>CE11-80bcd81982</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I55" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
           <t>11</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr">
+      <c r="K55" t="inlineStr">
         <is>
           <t>使用 CREATE INDEX 语句创建索引</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L55" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8323,42 +8671,47 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
           <t>使用 ALTER TABLE 语句
 添加索引</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="G56" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr">
+      <c r="H56" t="inlineStr">
         <is>
           <t>CE11-17839bf0fb</t>
         </is>
       </c>
-      <c r="H56" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I56" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
           <t>11</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr">
+      <c r="K56" t="inlineStr">
         <is>
           <t>使用 ALTER TABLE 语句
 添加索引</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L56" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8372,7 +8725,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CK015</t>
+          <t>CK060</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -8382,45 +8735,50 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>CREATE TABLE创建数据表</t>
+          <t>建表时定义索引</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
+          <t>建表语境中的索引定义；由原CK015出现记录迁移，不重复新增出现记录</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
           <t>在 CREATE TABLE 时通过约束或指定索引方式创建索引。</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="G57" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="H57" t="inlineStr">
         <is>
           <t>CE11-dcbb4b95a2</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I57" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
           <t>11</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr">
+      <c r="K57" t="inlineStr">
         <is>
           <t>在 CREATE TABLE 时通过约束或指定索引方式创建索引。</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L57" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8449,42 +8807,47 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
           <t>索引删
 除及维护</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="H58" t="inlineStr">
         <is>
           <t>CE11-c0aa5639a8</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I58" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
           <t>11</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr">
+      <c r="K58" t="inlineStr">
         <is>
           <t>索引删
 除及维护</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L58" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8513,42 +8876,47 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
           <t>引导
 学生对比有无索引的查询效果</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="G59" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="H59" t="inlineStr">
         <is>
           <t>CE11-eeed49a9bf</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I59" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
           <t>11</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr">
+      <c r="K59" t="inlineStr">
         <is>
           <t>引导
 学生对比有无索引的查询效果</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L59" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8577,42 +8945,47 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
           <t>数据备份与恢复的必要性。使用数据库工具或命令进行备份与恢复的基本操
 作流程。</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="H60" t="inlineStr">
         <is>
           <t>CE12-f64363af28</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I60" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr">
+      <c r="K60" t="inlineStr">
         <is>
           <t>数据备份与恢复的必要性。使用数据库工具或命令进行备份与恢复的基本操
 作流程。</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L60" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8641,40 +9014,45 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
           <t>事务的概念、ACID 特性（原子性、一致性、隔离性、持久性）</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="G61" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="H61" t="inlineStr">
         <is>
           <t>CE12-1c61fa29af</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I61" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr">
+      <c r="K61" t="inlineStr">
         <is>
           <t>事务的概念、ACID 特性（原子性、一致性、隔离性、持久性）</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L61" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
         <is>
           <t>待审查</t>
         </is>
@@ -8703,49 +9081,54 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
+          <t>沿用原文项目语境</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
           <t>事务
 控制语句（BEGIN, COMMIT, ROLLBACK）的使用。</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="G62" t="inlineStr">
         <is>
           <t>同一知识点跨项目共用CK，出现记录分别保留</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="H62" t="inlineStr">
         <is>
           <t>CE12-5215a91fe3</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>课标0913.pdf</t>
-        </is>
-      </c>
       <c r="I62" t="inlineStr">
         <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr">
+      <c r="K62" t="inlineStr">
         <is>
           <t>事务
 控制语句（BEGIN, COMMIT, ROLLBACK）的使用。</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
-        </is>
-      </c>
       <c r="L62" t="inlineStr">
         <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
           <t>待审查</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L62"/>
+  <autoFilter ref="A1:M62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9005,4 +9388,303 @@
   <autoFilter ref="A1:K4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>接口ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>知识点ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>项目ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>技术行为标签</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>学生操作要求</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>明确独立操作</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>关联教学活动ID</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>关联检查证据ID</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>判断边界</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>支持等级</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>标签来源</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>证据ID</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>来源文件名</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>PDF实际页码</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>原文摘录</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>来源状态</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>研究者审查状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CTB001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CK057</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>备份相关技术行为</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>独立完成备份实验</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>是，原文明示</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CA026</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>EC015;EC016</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>两标签来自同一组合句，未规定各自独立评分；不是同一岗位能力，也不构成教学先修</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>本轮不判定</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>研究组织；技术活动由原文支持</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>CE12-25ece1edeb;CE12-7b942d42b5</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>学生独立完成备份、恢复和事务操作实验
+——
+及时答疑纠错。</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>待审查</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CTB002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CK057</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>P08</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>恢复相关技术行为</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>独立完成恢复实验</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>是，原文明示</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CA026</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EC015;EC016</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>两标签来自同一组合句，未规定各自独立评分；不是同一岗位能力，也不构成教学先修</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>本轮不判定</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>研究组织；技术活动由原文支持</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>CE12-25ece1edeb;CE12-7b942d42b5</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>课标0913.pdf</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>学生独立完成备份、恢复和事务操作实验
+——
+及时答疑纠错。</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>可见正文文本层摘录；已作页面浏览，待研究者审查</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>待审查</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>